<commit_message>
Stage 8 review fixes: F-012
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/Development/OD23/Vehicle_Ladder/Bench_Sheets/OD23_dilution-check_092226_revA.xlsx
+++ b/output/archive/DurnesswickData/Development/OD23/Vehicle_Ladder/Bench_Sheets/OD23_dilution-check_092226_revA.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -903,11 +903,7 @@
           <t>1:10</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Settles, redispersible</t>
-        </is>
-      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Repeat pending</t>
@@ -986,38 +982,63 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Stock 1</t>
+          <t>Stock preparation</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>Drug stock in mg/ml</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Target in µM</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Equivalent in nM</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Unit check open</t>
+          <t>Check</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Stock 2</t>
+          <t>Source stock record</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Unit check open</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+    </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Temperature set by the client; value to be confirmed before the repeat is run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Initial settling/redispersion observations belong to the undiluted ladder. Dilution-repeat results remain blank.</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1097,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Units are mixed across the working sheets (mg/mL and mg/ml; µM and nM in the repeat stock table). Standardise to mg/mL and nM before the final sheet is issued.</t>
+          <t>Units are mixed across working sheets (mg/mL and mg/ml; µM and nM in the repeat template). Resolve the concentration basis before final issue; conversion between mass and molar units requires molecular weight.</t>
         </is>
       </c>
     </row>

</xml_diff>